<commit_message>
Update: combined campus names in filters and fixed admin authorization rules
</commit_message>
<xml_diff>
--- a/Uploader_Config.xlsx
+++ b/Uploader_Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Projects\ENGG Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{984A90C9-35DF-40BB-B8D0-4A8B92BBD62B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E85411FA-0C05-43E6-A02F-2050A914EDA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="3">
   <si>
     <t>Category</t>
   </si>
@@ -406,7 +406,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9782594E-49BA-43C6-9E7A-F1DB7B294A92}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:B56"/>
+  <dimension ref="A1:B248"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.625" customWidth="1"/>
@@ -423,7 +423,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>213309039</v>
+        <v>213309197</v>
       </c>
       <c r="B2" t="s">
         <v>1</v>
@@ -431,7 +431,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>213309050</v>
+        <v>235546175</v>
       </c>
       <c r="B3" t="s">
         <v>1</v>
@@ -439,7 +439,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>202308695</v>
+        <v>224308547</v>
       </c>
       <c r="B4" t="s">
         <v>1</v>
@@ -447,7 +447,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>224308372</v>
+        <v>213307925</v>
       </c>
       <c r="B5" t="s">
         <v>1</v>
@@ -455,7 +455,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>213309044</v>
+        <v>213307657</v>
       </c>
       <c r="B6" t="s">
         <v>1</v>
@@ -463,7 +463,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>246401089</v>
+        <v>213307647</v>
       </c>
       <c r="B7" t="s">
         <v>1</v>
@@ -471,7 +471,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>202308425</v>
+        <v>224308554</v>
       </c>
       <c r="B8" t="s">
         <v>1</v>
@@ -479,7 +479,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>202308763</v>
+        <v>213309207</v>
       </c>
       <c r="B9" t="s">
         <v>1</v>
@@ -487,7 +487,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>246400482</v>
+        <v>257403463</v>
       </c>
       <c r="B10" t="s">
         <v>1</v>
@@ -495,7 +495,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>202308788</v>
+        <v>257403475</v>
       </c>
       <c r="B11" t="s">
         <v>1</v>
@@ -503,7 +503,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>213307188</v>
+        <v>224308529</v>
       </c>
       <c r="B12" t="s">
         <v>1</v>
@@ -511,7 +511,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>202308745</v>
+        <v>235416087</v>
       </c>
       <c r="B13" t="s">
         <v>1</v>
@@ -519,7 +519,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>202308714</v>
+        <v>213307895</v>
       </c>
       <c r="B14" t="s">
         <v>1</v>
@@ -527,7 +527,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>202308728</v>
+        <v>224308620</v>
       </c>
       <c r="B15" t="s">
         <v>1</v>
@@ -535,7 +535,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>202308514</v>
+        <v>257400756</v>
       </c>
       <c r="B16" t="s">
         <v>1</v>
@@ -543,7 +543,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>202308520</v>
+        <v>224364920</v>
       </c>
       <c r="B17" t="s">
         <v>1</v>
@@ -551,7 +551,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>224308370</v>
+        <v>224308530</v>
       </c>
       <c r="B18" t="s">
         <v>1</v>
@@ -559,7 +559,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>246401403</v>
+        <v>257404447</v>
       </c>
       <c r="B19" t="s">
         <v>1</v>
@@ -567,7 +567,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>202308420</v>
+        <v>224308539</v>
       </c>
       <c r="B20" t="s">
         <v>1</v>
@@ -575,7 +575,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>246404571</v>
+        <v>235562276</v>
       </c>
       <c r="B21" t="s">
         <v>1</v>
@@ -583,7 +583,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>224364899</v>
+        <v>235562275</v>
       </c>
       <c r="B22" t="s">
         <v>1</v>
@@ -591,7 +591,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>246413511</v>
+        <v>257403799</v>
       </c>
       <c r="B23" t="s">
         <v>1</v>
@@ -599,7 +599,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>224308358</v>
+        <v>224364923</v>
       </c>
       <c r="B24" t="s">
         <v>1</v>
@@ -607,7 +607,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>213307191</v>
+        <v>224360533</v>
       </c>
       <c r="B25" t="s">
         <v>1</v>
@@ -615,7 +615,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>213307422</v>
+        <v>257402519</v>
       </c>
       <c r="B26" t="s">
         <v>1</v>
@@ -623,7 +623,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>246406555</v>
+        <v>224308517</v>
       </c>
       <c r="B27" t="s">
         <v>1</v>
@@ -631,7 +631,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>202309424</v>
+        <v>257403497</v>
       </c>
       <c r="B28" t="s">
         <v>1</v>
@@ -639,7 +639,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>202308528</v>
+        <v>257429737</v>
       </c>
       <c r="B29" t="s">
         <v>1</v>
@@ -647,7 +647,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>213309197</v>
+        <v>235546454</v>
       </c>
       <c r="B30" t="s">
         <v>1</v>
@@ -655,7 +655,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31">
-        <v>224308547</v>
+        <v>213307638</v>
       </c>
       <c r="B31" t="s">
         <v>1</v>
@@ -663,7 +663,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>213307657</v>
+        <v>257403496</v>
       </c>
       <c r="B32" t="s">
         <v>1</v>
@@ -671,7 +671,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>213307925</v>
+        <v>224308531</v>
       </c>
       <c r="B33" t="s">
         <v>1</v>
@@ -679,7 +679,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>224308538</v>
+        <v>235418547</v>
       </c>
       <c r="B34" t="s">
         <v>1</v>
@@ -687,7 +687,7 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>224308554</v>
+        <v>224308650</v>
       </c>
       <c r="B35" t="s">
         <v>1</v>
@@ -695,7 +695,7 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>213309207</v>
+        <v>235546691</v>
       </c>
       <c r="B36" t="s">
         <v>1</v>
@@ -703,7 +703,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>257403463</v>
+        <v>257405136</v>
       </c>
       <c r="B37" t="s">
         <v>1</v>
@@ -711,7 +711,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38">
-        <v>224364920</v>
+        <v>235416351</v>
       </c>
       <c r="B38" t="s">
         <v>1</v>
@@ -719,7 +719,7 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39">
-        <v>213307850</v>
+        <v>235562284</v>
       </c>
       <c r="B39" t="s">
         <v>1</v>
@@ -727,7 +727,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40">
-        <v>224308539</v>
+        <v>213309193</v>
       </c>
       <c r="B40" t="s">
         <v>1</v>
@@ -735,7 +735,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41">
-        <v>235562276</v>
+        <v>213309272</v>
       </c>
       <c r="B41" t="s">
         <v>1</v>
@@ -743,7 +743,7 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42">
-        <v>235416087</v>
+        <v>235419904</v>
       </c>
       <c r="B42" t="s">
         <v>1</v>
@@ -751,7 +751,7 @@
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43">
-        <v>224308529</v>
+        <v>213309202</v>
       </c>
       <c r="B43" t="s">
         <v>1</v>
@@ -759,7 +759,7 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44">
-        <v>213307647</v>
+        <v>235546167</v>
       </c>
       <c r="B44" t="s">
         <v>1</v>
@@ -767,7 +767,7 @@
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45">
-        <v>235547954</v>
+        <v>235416971</v>
       </c>
       <c r="B45" t="s">
         <v>1</v>
@@ -775,7 +775,7 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46">
-        <v>213307638</v>
+        <v>235416653</v>
       </c>
       <c r="B46" t="s">
         <v>1</v>
@@ -783,7 +783,7 @@
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47">
-        <v>213307648</v>
+        <v>224308664</v>
       </c>
       <c r="B47" t="s">
         <v>1</v>
@@ -791,7 +791,7 @@
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48">
-        <v>213309275</v>
+        <v>213309271</v>
       </c>
       <c r="B48" t="s">
         <v>1</v>
@@ -799,7 +799,7 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49">
-        <v>213309763</v>
+        <v>235546535</v>
       </c>
       <c r="B49" t="s">
         <v>1</v>
@@ -807,7 +807,7 @@
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>213309287</v>
+        <v>224308538</v>
       </c>
       <c r="B50" t="s">
         <v>1</v>
@@ -815,7 +815,7 @@
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>235562284</v>
+        <v>257404490</v>
       </c>
       <c r="B51" t="s">
         <v>1</v>
@@ -823,7 +823,7 @@
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52">
-        <v>235416653</v>
+        <v>224308528</v>
       </c>
       <c r="B52" t="s">
         <v>1</v>
@@ -831,7 +831,7 @@
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53">
-        <v>235546175</v>
+        <v>257403809</v>
       </c>
       <c r="B53" t="s">
         <v>1</v>
@@ -839,7 +839,7 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54">
-        <v>213307895</v>
+        <v>213309188</v>
       </c>
       <c r="B54" t="s">
         <v>1</v>
@@ -847,7 +847,7 @@
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55">
-        <v>235545017</v>
+        <v>235416115</v>
       </c>
       <c r="B55" t="s">
         <v>1</v>
@@ -855,9 +855,1545 @@
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56">
-        <v>235545018</v>
+        <v>257400813</v>
       </c>
       <c r="B56" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>257428936</v>
+      </c>
+      <c r="B57" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>224308743</v>
+      </c>
+      <c r="B58" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>235546580</v>
+      </c>
+      <c r="B59" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>213307642</v>
+      </c>
+      <c r="B60" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>224308567</v>
+      </c>
+      <c r="B61" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>235547954</v>
+      </c>
+      <c r="B62" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>257407052</v>
+      </c>
+      <c r="B63" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>224308545</v>
+      </c>
+      <c r="B64" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>257407038</v>
+      </c>
+      <c r="B65" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>213307634</v>
+      </c>
+      <c r="B66" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>235416067</v>
+      </c>
+      <c r="B67" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>224308525</v>
+      </c>
+      <c r="B68" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>224308520</v>
+      </c>
+      <c r="B69" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>213309199</v>
+      </c>
+      <c r="B70" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>224308666</v>
+      </c>
+      <c r="B71" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>246553606</v>
+      </c>
+      <c r="B72" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>213307900</v>
+      </c>
+      <c r="B73" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>224308507</v>
+      </c>
+      <c r="B74" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>213307648</v>
+      </c>
+      <c r="B75" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>213309287</v>
+      </c>
+      <c r="B76" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>257403803</v>
+      </c>
+      <c r="B77" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>213309763</v>
+      </c>
+      <c r="B78" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>213307632</v>
+      </c>
+      <c r="B79" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>213307650</v>
+      </c>
+      <c r="B80" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>235418579</v>
+      </c>
+      <c r="B81" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>257401484</v>
+      </c>
+      <c r="B82" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>257403505</v>
+      </c>
+      <c r="B83" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>257403494</v>
+      </c>
+      <c r="B84" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>257400093</v>
+      </c>
+      <c r="B85" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>257403476</v>
+      </c>
+      <c r="B86" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>235546471</v>
+      </c>
+      <c r="B87" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>235417242</v>
+      </c>
+      <c r="B88" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>235546973</v>
+      </c>
+      <c r="B89" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>257403503</v>
+      </c>
+      <c r="B90" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>257404458</v>
+      </c>
+      <c r="B91" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>235419634</v>
+      </c>
+      <c r="B92" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>235417003</v>
+      </c>
+      <c r="B93" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>235419747</v>
+      </c>
+      <c r="B94" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>257409579</v>
+      </c>
+      <c r="B95" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>257407044</v>
+      </c>
+      <c r="B96" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>224308534</v>
+      </c>
+      <c r="B97" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>257403789</v>
+      </c>
+      <c r="B98" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>257402938</v>
+      </c>
+      <c r="B99" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>257405725</v>
+      </c>
+      <c r="B100" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>257402249</v>
+      </c>
+      <c r="B101" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A102">
+        <v>213307651</v>
+      </c>
+      <c r="B102" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A103">
+        <v>268405681</v>
+      </c>
+      <c r="B103" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A104">
+        <v>257407043</v>
+      </c>
+      <c r="B104" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A105">
+        <v>213309187</v>
+      </c>
+      <c r="B105" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A106">
+        <v>257402241</v>
+      </c>
+      <c r="B106" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A107">
+        <v>257403768</v>
+      </c>
+      <c r="B107" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A108">
+        <v>257400746</v>
+      </c>
+      <c r="B108" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A109">
+        <v>257405740</v>
+      </c>
+      <c r="B109" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A110">
+        <v>213307926</v>
+      </c>
+      <c r="B110" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A111">
+        <v>213309210</v>
+      </c>
+      <c r="B111" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A112">
+        <v>235416138</v>
+      </c>
+      <c r="B112" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A113">
+        <v>257401255</v>
+      </c>
+      <c r="B113" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A114">
+        <v>235546191</v>
+      </c>
+      <c r="B114" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A115">
+        <v>257403460</v>
+      </c>
+      <c r="B115" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A116">
+        <v>235419459</v>
+      </c>
+      <c r="B116" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A117">
+        <v>235419923</v>
+      </c>
+      <c r="B117" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A118">
+        <v>257402520</v>
+      </c>
+      <c r="B118" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A119">
+        <v>235549308</v>
+      </c>
+      <c r="B119" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A120">
+        <v>213309184</v>
+      </c>
+      <c r="B120" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A121">
+        <v>235562471</v>
+      </c>
+      <c r="B121" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A122">
+        <v>257405355</v>
+      </c>
+      <c r="B122" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A123">
+        <v>213307652</v>
+      </c>
+      <c r="B123" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A124">
+        <v>224308543</v>
+      </c>
+      <c r="B124" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A125">
+        <v>224308546</v>
+      </c>
+      <c r="B125" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A126">
+        <v>257408327</v>
+      </c>
+      <c r="B126" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A127">
+        <v>257404461</v>
+      </c>
+      <c r="B127" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A128">
+        <v>213307617</v>
+      </c>
+      <c r="B128" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A129">
+        <v>257403970</v>
+      </c>
+      <c r="B129" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A130">
+        <v>224308508</v>
+      </c>
+      <c r="B130" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A131">
+        <v>257401481</v>
+      </c>
+      <c r="B131" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A132">
+        <v>213307654</v>
+      </c>
+      <c r="B132" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A133">
+        <v>213309201</v>
+      </c>
+      <c r="B133" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A134">
+        <v>257403469</v>
+      </c>
+      <c r="B134" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A135">
+        <v>224308544</v>
+      </c>
+      <c r="B135" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A136">
+        <v>257401733</v>
+      </c>
+      <c r="B136" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A137">
+        <v>257400322</v>
+      </c>
+      <c r="B137" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A138">
+        <v>246410694</v>
+      </c>
+      <c r="B138" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A139">
+        <v>257426041</v>
+      </c>
+      <c r="B139" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A140">
+        <v>235416346</v>
+      </c>
+      <c r="B140" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A141">
+        <v>257403489</v>
+      </c>
+      <c r="B141" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A142">
+        <v>224308709</v>
+      </c>
+      <c r="B142" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A143">
+        <v>257405137</v>
+      </c>
+      <c r="B143" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A144">
+        <v>257418289</v>
+      </c>
+      <c r="B144" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A145">
+        <v>235546298</v>
+      </c>
+      <c r="B145" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A146">
+        <v>257403793</v>
+      </c>
+      <c r="B146" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A147">
+        <v>257405103</v>
+      </c>
+      <c r="B147" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A148">
+        <v>257405119</v>
+      </c>
+      <c r="B148" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A149">
+        <v>257418273</v>
+      </c>
+      <c r="B149" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A150">
+        <v>213309195</v>
+      </c>
+      <c r="B150" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A151">
+        <v>213307850</v>
+      </c>
+      <c r="B151" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A152">
+        <v>224308535</v>
+      </c>
+      <c r="B152" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A153">
+        <v>257403470</v>
+      </c>
+      <c r="B153" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A154">
+        <v>257403770</v>
+      </c>
+      <c r="B154" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A155">
+        <v>213309200</v>
+      </c>
+      <c r="B155" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A156">
+        <v>213307656</v>
+      </c>
+      <c r="B156" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A157">
+        <v>257402321</v>
+      </c>
+      <c r="B157" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A158">
+        <v>235419804</v>
+      </c>
+      <c r="B158" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A159">
+        <v>257418595</v>
+      </c>
+      <c r="B159" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A160">
+        <v>235419423</v>
+      </c>
+      <c r="B160" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A161">
+        <v>224308540</v>
+      </c>
+      <c r="B161" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A162">
+        <v>257402320</v>
+      </c>
+      <c r="B162" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A163">
+        <v>257405736</v>
+      </c>
+      <c r="B163" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A164">
+        <v>257400758</v>
+      </c>
+      <c r="B164" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A165">
+        <v>257403492</v>
+      </c>
+      <c r="B165" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A166">
+        <v>257401285</v>
+      </c>
+      <c r="B166" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A167">
+        <v>213309186</v>
+      </c>
+      <c r="B167" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A168">
+        <v>213307639</v>
+      </c>
+      <c r="B168" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A169">
+        <v>257406380</v>
+      </c>
+      <c r="B169" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A170">
+        <v>257405721</v>
+      </c>
+      <c r="B170" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A171">
+        <v>257404462</v>
+      </c>
+      <c r="B171" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A172">
+        <v>257403808</v>
+      </c>
+      <c r="B172" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A173">
+        <v>224308524</v>
+      </c>
+      <c r="B173" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A174">
+        <v>224308523</v>
+      </c>
+      <c r="B174" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A175">
+        <v>224308654</v>
+      </c>
+      <c r="B175" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A176">
+        <v>257403465</v>
+      </c>
+      <c r="B176" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A177">
+        <v>257400510</v>
+      </c>
+      <c r="B177" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A178">
+        <v>224308606</v>
+      </c>
+      <c r="B178" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A179">
+        <v>257402526</v>
+      </c>
+      <c r="B179" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A180">
+        <v>235546161</v>
+      </c>
+      <c r="B180" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A181">
+        <v>224308537</v>
+      </c>
+      <c r="B181" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A182">
+        <v>235418514</v>
+      </c>
+      <c r="B182" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A183">
+        <v>257403453</v>
+      </c>
+      <c r="B183" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A184">
+        <v>257402924</v>
+      </c>
+      <c r="B184" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A185">
+        <v>224308557</v>
+      </c>
+      <c r="B185" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A186">
+        <v>257404445</v>
+      </c>
+      <c r="B186" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A187">
+        <v>257400316</v>
+      </c>
+      <c r="B187" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A188">
+        <v>235546297</v>
+      </c>
+      <c r="B188" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A189">
+        <v>224308592</v>
+      </c>
+      <c r="B189" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A190">
+        <v>257414538</v>
+      </c>
+      <c r="B190" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A191">
+        <v>235546373</v>
+      </c>
+      <c r="B191" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A192">
+        <v>224308602</v>
+      </c>
+      <c r="B192" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A193">
+        <v>213309288</v>
+      </c>
+      <c r="B193" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A194">
+        <v>224308533</v>
+      </c>
+      <c r="B194" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A195">
+        <v>257400324</v>
+      </c>
+      <c r="B195" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A196">
+        <v>235419504</v>
+      </c>
+      <c r="B196" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A197">
+        <v>235419503</v>
+      </c>
+      <c r="B197" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A198">
+        <v>224364921</v>
+      </c>
+      <c r="B198" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A199">
+        <v>213309283</v>
+      </c>
+      <c r="B199" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A200">
+        <v>213309276</v>
+      </c>
+      <c r="B200" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A201">
+        <v>257403796</v>
+      </c>
+      <c r="B201" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A202">
+        <v>213309284</v>
+      </c>
+      <c r="B202" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A203">
+        <v>224308553</v>
+      </c>
+      <c r="B203" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A204">
+        <v>257408950</v>
+      </c>
+      <c r="B204" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A205">
+        <v>257406385</v>
+      </c>
+      <c r="B205" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A206">
+        <v>257403500</v>
+      </c>
+      <c r="B206" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A207">
+        <v>246411657</v>
+      </c>
+      <c r="B207" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A208">
+        <v>257400315</v>
+      </c>
+      <c r="B208" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A209">
+        <v>257404484</v>
+      </c>
+      <c r="B209" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A210">
+        <v>257406243</v>
+      </c>
+      <c r="B210" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A211">
+        <v>257410201</v>
+      </c>
+      <c r="B211" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A212">
+        <v>257405096</v>
+      </c>
+      <c r="B212" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A213">
+        <v>257400167</v>
+      </c>
+      <c r="B213" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A214">
+        <v>235545270</v>
+      </c>
+      <c r="B214" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A215">
+        <v>213307649</v>
+      </c>
+      <c r="B215" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A216">
+        <v>224308559</v>
+      </c>
+      <c r="B216" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A217">
+        <v>224308549</v>
+      </c>
+      <c r="B217" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A218">
+        <v>224308536</v>
+      </c>
+      <c r="B218" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A219">
+        <v>257403509</v>
+      </c>
+      <c r="B219" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A220">
+        <v>257406395</v>
+      </c>
+      <c r="B220" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A221">
+        <v>235419777</v>
+      </c>
+      <c r="B221" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A222">
+        <v>213309183</v>
+      </c>
+      <c r="B222" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A223">
+        <v>257405731</v>
+      </c>
+      <c r="B223" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A224">
+        <v>257404621</v>
+      </c>
+      <c r="B224" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A225">
+        <v>257409582</v>
+      </c>
+      <c r="B225" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A226">
+        <v>257407055</v>
+      </c>
+      <c r="B226" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A227">
+        <v>257419315</v>
+      </c>
+      <c r="B227" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A228">
+        <v>224308597</v>
+      </c>
+      <c r="B228" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A229">
+        <v>257410200</v>
+      </c>
+      <c r="B229" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A230">
+        <v>257403478</v>
+      </c>
+      <c r="B230" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A231">
+        <v>257408326</v>
+      </c>
+      <c r="B231" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A232">
+        <v>235417875</v>
+      </c>
+      <c r="B232" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A233">
+        <v>235546168</v>
+      </c>
+      <c r="B233" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A234">
+        <v>224308599</v>
+      </c>
+      <c r="B234" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A235">
+        <v>213309761</v>
+      </c>
+      <c r="B235" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A236">
+        <v>235552252</v>
+      </c>
+      <c r="B236" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A237">
+        <v>224308601</v>
+      </c>
+      <c r="B237" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="238" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A238">
+        <v>257420379</v>
+      </c>
+      <c r="B238" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="239" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A239">
+        <v>235418564</v>
+      </c>
+      <c r="B239" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A240">
+        <v>224308598</v>
+      </c>
+      <c r="B240" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A241">
+        <v>224308603</v>
+      </c>
+      <c r="B241" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A242">
+        <v>246414358</v>
+      </c>
+      <c r="B242" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A243">
+        <v>257405348</v>
+      </c>
+      <c r="B243" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A244">
+        <v>224308518</v>
+      </c>
+      <c r="B244" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A245">
+        <v>257406390</v>
+      </c>
+      <c r="B245" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A246">
+        <v>257405127</v>
+      </c>
+      <c r="B246" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A247">
+        <v>257428631</v>
+      </c>
+      <c r="B247" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A248">
+        <v>257382811</v>
+      </c>
+      <c r="B248" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>